<commit_message>
Modif fichier Suivi version algo
</commit_message>
<xml_diff>
--- a/Suivi_Version_AlgoCNN.xlsx
+++ b/Suivi_Version_AlgoCNN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjdia\Desktop\TSE\SCOT - Projet Innovation\scot-projet-innovation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16d0ed9cc9be81b2/Documents/TSE/Projet Innovation/scot-projet-innovation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3B027D9-9D59-48BD-9498-914684CDC09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{A3B027D9-9D59-48BD-9498-914684CDC09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50AF5517-FC5B-4365-877A-5059884F948F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{60EBD7B7-60BA-44E1-BC6B-0954BE402623}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{60EBD7B7-60BA-44E1-BC6B-0954BE402623}"/>
   </bookViews>
   <sheets>
     <sheet name="Synthèse" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="116">
   <si>
     <t>Nb EPOCH</t>
   </si>
@@ -60,13 +60,340 @@
   </si>
   <si>
     <t>Version Algo CNN</t>
+  </si>
+  <si>
+    <t>Premiere version issu de claude</t>
+  </si>
+  <si>
+    <t>simule l'irrégularité des inclusions + penalisation des erreurs inclusions</t>
+  </si>
+  <si>
+    <t>suppression pénalisation des erreurs inclusion</t>
+  </si>
+  <si>
+    <t>Epoch</t>
+  </si>
+  <si>
+    <t>Train Loss</t>
+  </si>
+  <si>
+    <t>Train Acc</t>
+  </si>
+  <si>
+    <t>Val Loss</t>
+  </si>
+  <si>
+    <t>Val Acc</t>
+  </si>
+  <si>
+    <t>0.9323</t>
+  </si>
+  <si>
+    <t>52.8%</t>
+  </si>
+  <si>
+    <t>1.0109</t>
+  </si>
+  <si>
+    <t>55.6%</t>
+  </si>
+  <si>
+    <t>0.8485</t>
+  </si>
+  <si>
+    <t>53.2%</t>
+  </si>
+  <si>
+    <t>0.6701</t>
+  </si>
+  <si>
+    <t>57.8%</t>
+  </si>
+  <si>
+    <t>0.7770</t>
+  </si>
+  <si>
+    <t>58.8%</t>
+  </si>
+  <si>
+    <t>0.9081</t>
+  </si>
+  <si>
+    <t>57.2%</t>
+  </si>
+  <si>
+    <t>0.7160</t>
+  </si>
+  <si>
+    <t>61.0%</t>
+  </si>
+  <si>
+    <t>0.6050</t>
+  </si>
+  <si>
+    <t>69.4%</t>
+  </si>
+  <si>
+    <t>0.6898</t>
+  </si>
+  <si>
+    <t>62.4%</t>
+  </si>
+  <si>
+    <t>0.5416</t>
+  </si>
+  <si>
+    <t>77.8%</t>
+  </si>
+  <si>
+    <t>0.7526</t>
+  </si>
+  <si>
+    <t>64.2%</t>
+  </si>
+  <si>
+    <t>0.5761</t>
+  </si>
+  <si>
+    <t>66.7%</t>
+  </si>
+  <si>
+    <t>0.7270</t>
+  </si>
+  <si>
+    <t>65.0%</t>
+  </si>
+  <si>
+    <t>0.5720</t>
+  </si>
+  <si>
+    <t>72.8%</t>
+  </si>
+  <si>
+    <t>0.7121</t>
+  </si>
+  <si>
+    <t>64.6%</t>
+  </si>
+  <si>
+    <t>0.4778</t>
+  </si>
+  <si>
+    <t>76.7%</t>
+  </si>
+  <si>
+    <t>0.7061</t>
+  </si>
+  <si>
+    <t>63.6%</t>
+  </si>
+  <si>
+    <t>0.5876</t>
+  </si>
+  <si>
+    <t>74.4%</t>
+  </si>
+  <si>
+    <t>0.6825</t>
+  </si>
+  <si>
+    <t>0.4858</t>
+  </si>
+  <si>
+    <t>76.1%</t>
+  </si>
+  <si>
+    <t>0.6963</t>
+  </si>
+  <si>
+    <t>67.4%</t>
+  </si>
+  <si>
+    <t>0.5496</t>
+  </si>
+  <si>
+    <t>75.6%</t>
+  </si>
+  <si>
+    <t>0.6380</t>
+  </si>
+  <si>
+    <t>71.8%</t>
+  </si>
+  <si>
+    <t>0.4093</t>
+  </si>
+  <si>
+    <t>86.1%</t>
+  </si>
+  <si>
+    <t>0.6466</t>
+  </si>
+  <si>
+    <t>69.9%</t>
+  </si>
+  <si>
+    <t>0.4591</t>
+  </si>
+  <si>
+    <t>83.3%</t>
+  </si>
+  <si>
+    <t>0.6332</t>
+  </si>
+  <si>
+    <t>71.1%</t>
+  </si>
+  <si>
+    <t>0.4754</t>
+  </si>
+  <si>
+    <t>81.1%</t>
+  </si>
+  <si>
+    <t>0.6037</t>
+  </si>
+  <si>
+    <t>74.0%</t>
+  </si>
+  <si>
+    <t>0.3946</t>
+  </si>
+  <si>
+    <t>88.3%</t>
+  </si>
+  <si>
+    <t>0.6389</t>
+  </si>
+  <si>
+    <t>0.4873</t>
+  </si>
+  <si>
+    <t>0.6162</t>
+  </si>
+  <si>
+    <t>69.7%</t>
+  </si>
+  <si>
+    <t>0.3758</t>
+  </si>
+  <si>
+    <t>87.2%</t>
+  </si>
+  <si>
+    <t>0.6002</t>
+  </si>
+  <si>
+    <t>74.2%</t>
+  </si>
+  <si>
+    <t>0.4041</t>
+  </si>
+  <si>
+    <t>0.6200</t>
+  </si>
+  <si>
+    <t>73.8%</t>
+  </si>
+  <si>
+    <t>0.4063</t>
+  </si>
+  <si>
+    <t>0.5717</t>
+  </si>
+  <si>
+    <t>0.4124</t>
+  </si>
+  <si>
+    <t>85.0%</t>
+  </si>
+  <si>
+    <t>0.6145</t>
+  </si>
+  <si>
+    <t>0.3952</t>
+  </si>
+  <si>
+    <t>87.8%</t>
+  </si>
+  <si>
+    <t>0.5381</t>
+  </si>
+  <si>
+    <t>76.2%</t>
+  </si>
+  <si>
+    <t>0.3569</t>
+  </si>
+  <si>
+    <t>0.6262</t>
+  </si>
+  <si>
+    <t>73.2%</t>
+  </si>
+  <si>
+    <t>0.3933</t>
+  </si>
+  <si>
+    <t>0.5868</t>
+  </si>
+  <si>
+    <t>72.9%</t>
+  </si>
+  <si>
+    <t>0.3766</t>
+  </si>
+  <si>
+    <t>0.5401</t>
+  </si>
+  <si>
+    <t>75.3%</t>
+  </si>
+  <si>
+    <t>0.3649</t>
+  </si>
+  <si>
+    <t>0.5409</t>
+  </si>
+  <si>
+    <t>0.3639</t>
+  </si>
+  <si>
+    <t>0.5505</t>
+  </si>
+  <si>
+    <t>0.3602</t>
+  </si>
+  <si>
+    <t>0.5915</t>
+  </si>
+  <si>
+    <t>0.3618</t>
+  </si>
+  <si>
+    <t>0.5568</t>
+  </si>
+  <si>
+    <t>75.1%</t>
+  </si>
+  <si>
+    <t>0.3623</t>
+  </si>
+  <si>
+    <t>0.5764</t>
+  </si>
+  <si>
+    <t>76.5%</t>
+  </si>
+  <si>
+    <t>0.3705</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +413,14 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -123,18 +458,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -470,7 +808,7 @@
   <dimension ref="B2:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -511,7 +849,9 @@
       <c r="C4" s="1">
         <v>30</v>
       </c>
-      <c r="D4" s="1"/>
+      <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -523,7 +863,9 @@
       <c r="C5" s="1">
         <v>30</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -535,7 +877,9 @@
       <c r="C6" s="1">
         <v>30</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -646,9 +990,537 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C3FFD5-4B48-45E2-89DB-6E50E94738FC}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B19">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" t="s">
+        <v>82</v>
+      </c>
+      <c r="F19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B20">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B21">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B22">
+        <v>21</v>
+      </c>
+      <c r="C22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B23">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B24">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>95</v>
+      </c>
+      <c r="D24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" t="s">
+        <v>97</v>
+      </c>
+      <c r="F24" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B25">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" t="s">
+        <v>100</v>
+      </c>
+      <c r="F25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B26">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" t="s">
+        <v>102</v>
+      </c>
+      <c r="E26" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B27">
+        <v>26</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" t="s">
+        <v>105</v>
+      </c>
+      <c r="F27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B28">
+        <v>27</v>
+      </c>
+      <c r="C28" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" t="s">
+        <v>107</v>
+      </c>
+      <c r="F28" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B29">
+        <v>28</v>
+      </c>
+      <c r="C29" t="s">
+        <v>108</v>
+      </c>
+      <c r="D29" t="s">
+        <v>50</v>
+      </c>
+      <c r="E29" t="s">
+        <v>109</v>
+      </c>
+      <c r="F29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B30">
+        <v>29</v>
+      </c>
+      <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" t="s">
+        <v>111</v>
+      </c>
+      <c r="E30" t="s">
+        <v>112</v>
+      </c>
+      <c r="F30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="B31">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>113</v>
+      </c>
+      <c r="D31" t="s">
+        <v>114</v>
+      </c>
+      <c r="E31" t="s">
+        <v>115</v>
+      </c>
+      <c r="F31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Version 3 du code
</commit_message>
<xml_diff>
--- a/Suivi_Version_AlgoCNN.xlsx
+++ b/Suivi_Version_AlgoCNN.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/16d0ed9cc9be81b2/Documents/TSE/Projet Innovation/scot-projet-innovation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tanka\Documents\Telecom\Projet Innovation\scot-projet-innovation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{A3B027D9-9D59-48BD-9498-914684CDC09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50AF5517-FC5B-4365-877A-5059884F948F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12537933-5A52-4FC4-B94C-15DDC71CDFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{60EBD7B7-60BA-44E1-BC6B-0954BE402623}"/>
+    <workbookView xWindow="2175" yWindow="1575" windowWidth="19950" windowHeight="9360" activeTab="3" xr2:uid="{60EBD7B7-60BA-44E1-BC6B-0954BE402623}"/>
   </bookViews>
   <sheets>
     <sheet name="Synthèse" sheetId="1" r:id="rId1"/>
@@ -30,8 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -39,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="148">
   <si>
     <t>Nb EPOCH</t>
   </si>
@@ -387,6 +385,102 @@
   </si>
   <si>
     <t>0.3705</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Epoch  Train Loss  Train Acc  Val Loss  Val Acc</t>
+  </si>
+  <si>
+    <t>───────────────────────────────────────────────────────</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     1      1.0486     41.0%    1.1122   33.3% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     2      0.8747     54.4%    1.0688   51.7% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     3      0.8426     52.9%    1.1126   57.2% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     4      0.7356     61.9%    0.7307   76.1% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     5      0.7314     63.7%    0.5920   80.6% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     6      0.7002     64.7%    0.5371   81.7% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     7      0.6856     65.8%    0.5134   81.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     8      0.7457     64.3%    0.6714   78.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     9      0.6857     68.1%    0.5502   80.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    10      0.6520     69.9%    0.6439   66.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    11      0.6767     69.3%    0.8475   66.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    12      0.6828     69.6%    0.4692   83.3% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    13      0.6469     69.4%    0.5711   68.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    14      0.6329     71.1%    0.4464   80.0%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    15      0.6408     71.1%    0.4914   85.0% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    16      0.6111     71.8%    0.4952   78.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    17      0.5994     72.5%    0.4376   83.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    18      0.6051     71.2%    0.4375   84.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    19      0.6271     74.2%    0.4150   85.6% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    20      0.6204     72.1%    0.3786   87.8% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    21      0.5928     75.3%    0.3718   86.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    22      0.5678     74.3%    0.3926   86.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    23      0.6054     76.2%    0.3830   88.9% ★</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    24      0.5884     76.4%    0.3828   88.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    25      0.5610     74.7%    0.3783   87.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    26      0.5752     75.4%    0.3771   87.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    27      0.5513     74.9%    0.3802   87.8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    28      0.5472     75.7%    0.3777   86.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    29      0.5753     75.3%    0.3822   84.4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    30      0.5369     78.5%    0.3827   84.4%</t>
   </si>
 </sst>
 </file>
@@ -466,10 +560,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -806,23 +900,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606DFC93-FC1B-41F9-8AC0-E265823407AC}">
   <dimension ref="B2:G18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="58.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="58.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="2:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-    </row>
-    <row r="3" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -842,7 +936,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>1</v>
       </c>
@@ -856,7 +950,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:7" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>2</v>
       </c>
@@ -870,21 +964,21 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>3</v>
       </c>
       <c r="C6" s="1">
         <v>30</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -892,7 +986,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -900,7 +994,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -908,7 +1002,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -916,7 +1010,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -924,7 +1018,7 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -932,7 +1026,7 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -940,7 +1034,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -948,7 +1042,7 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -956,7 +1050,7 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -964,7 +1058,7 @@
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -972,7 +1066,7 @@
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -991,9 +1085,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C3FFD5-4B48-45E2-89DB-6E50E94738FC}">
   <dimension ref="B1:F31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>10</v>
       </c>
@@ -1010,7 +1104,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2">
         <v>1</v>
       </c>
@@ -1027,7 +1121,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>2</v>
       </c>
@@ -1044,7 +1138,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>3</v>
       </c>
@@ -1061,7 +1155,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>4</v>
       </c>
@@ -1078,7 +1172,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>5</v>
       </c>
@@ -1095,7 +1189,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>6</v>
       </c>
@@ -1112,7 +1206,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>7</v>
       </c>
@@ -1129,7 +1223,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>8</v>
       </c>
@@ -1146,7 +1240,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>9</v>
       </c>
@@ -1163,7 +1257,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>10</v>
       </c>
@@ -1180,7 +1274,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>11</v>
       </c>
@@ -1197,7 +1291,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>12</v>
       </c>
@@ -1214,7 +1308,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>13</v>
       </c>
@@ -1231,7 +1325,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>14</v>
       </c>
@@ -1248,7 +1342,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>15</v>
       </c>
@@ -1265,7 +1359,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>16</v>
       </c>
@@ -1282,7 +1376,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>17</v>
       </c>
@@ -1299,7 +1393,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>18</v>
       </c>
@@ -1316,7 +1410,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>19</v>
       </c>
@@ -1333,7 +1427,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>20</v>
       </c>
@@ -1350,7 +1444,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>21</v>
       </c>
@@ -1367,7 +1461,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>22</v>
       </c>
@@ -1384,7 +1478,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>23</v>
       </c>
@@ -1401,7 +1495,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>24</v>
       </c>
@@ -1418,7 +1512,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>25</v>
       </c>
@@ -1435,7 +1529,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>26</v>
       </c>
@@ -1452,7 +1546,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>27</v>
       </c>
@@ -1469,7 +1563,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>28</v>
       </c>
@@ -1486,7 +1580,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30">
         <v>29</v>
       </c>
@@ -1503,7 +1597,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>30</v>
       </c>
@@ -1528,7 +1622,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F96A8959-4B07-4D3B-9340-0FA707C3646B}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1536,9 +1630,170 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE317CF4-B2A9-4E00-AA68-8275A4CDD8F8}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <dimension ref="B2:B33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B31" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>147</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout des images des output dans le Excel pour version 3 avec utilisation du GPU
</commit_message>
<xml_diff>
--- a/Suivi_Version_AlgoCNN.xlsx
+++ b/Suivi_Version_AlgoCNN.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tanka\Documents\Telecom\Projet Innovation\scot-projet-innovation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12537933-5A52-4FC4-B94C-15DDC71CDFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C3F6C9-ECC6-41C5-AF08-8F72E5E71F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2175" yWindow="1575" windowWidth="19950" windowHeight="9360" activeTab="3" xr2:uid="{60EBD7B7-60BA-44E1-BC6B-0954BE402623}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{60EBD7B7-60BA-44E1-BC6B-0954BE402623}"/>
   </bookViews>
   <sheets>
     <sheet name="Synthèse" sheetId="1" r:id="rId1"/>
@@ -580,6 +580,111 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>733425</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>476973</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>175653</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90BCBB26-7DD4-6C47-0270-2F511746955B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5305425" y="476250"/>
+          <a:ext cx="5077548" cy="4461903"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>194174</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>118579</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Image 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DB555A4-0297-4D89-93C5-FB39FC023B1A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5334000" y="5334000"/>
+          <a:ext cx="10862174" cy="3547579"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1795,5 +1900,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>